<commit_message>
Split company and template settings, add company logo and colors, redesign menu (SPEC-007)
- Menu: groups are named in sentence case under a hairline that stays when the
  sidebar collapses, so nothing wraps or jumps; the sidebar is 256 px so no label
  is cut. Administración lists Usuarios, Plantilla and Empresa.
- "Empresa y plantilla" becomes Empresa (/company) and Plantilla (/template).
  Each page saves only its own fields; the old link redirects to Empresa.
- "Firma" becomes "Representante legal"; the acceptance block prints the name,
  the title and the legal name, leaving out what is empty.
- Company logo (PNG or JPEG, validated and stored in SQLite, migration 007) and
  main color, edited in "Logo y colores" with a live preview of the quote header
  and color suggestions taken from the logo. The PDF and the workbook use them,
  and print the trade name when there is no logo.
- SPEC-007 records the decisions and the parts of SPEC-006 it supersedes.
</commit_message>
<xml_diff>
--- a/web/tests/fixtures/quote-document-A1.xlsx
+++ b/web/tests/fixtures/quote-document-A1.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="81">
   <si>
     <t>COTIZACIÓN</t>
   </si>
@@ -168,9 +168,6 @@
   </si>
   <si>
     <t>ACEPTACIÓN</t>
-  </si>
-  <si>
-    <t>CleanCode</t>
   </si>
   <si>
     <t>Aceptado por: Hospital Ejemplo S.A.</t>
@@ -324,7 +321,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="EEF2FF"/>
+        <fgColor rgb="EDEDFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -419,7 +416,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1981200" cy="373388"/>
+    <xdr:ext cx="1981200" cy="373951"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -1289,12 +1286,12 @@
     <row r="56" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" ht="25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
       <c r="D57" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E57" s="14"/>
       <c r="F57" s="14"/>
@@ -1304,7 +1301,7 @@
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
@@ -1385,132 +1382,132 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="D2" s="7">
         <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F2" s="6">
         <v>30</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="D3" s="7">
         <v>12</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F3" s="6">
         <v>30</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="D4" s="7">
         <v>120</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F4" s="6">
         <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D5" s="7">
         <v>80</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F5" s="6">
         <v>22</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>